<commit_message>
Excel con 4 hojas: Resumen, Historico, Modelo, Inputs
</commit_message>
<xml_diff>
--- a/artifacts/proyeccion_costos.xlsx
+++ b/artifacts/proyeccion_costos.xlsx
@@ -7,7 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Proyeccion" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Resumen" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Historico" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Modelo" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Inputs" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16,10 +19,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="$#,##0.00"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,27 +31,13 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b val="1"/>
-      <sz val="14"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="12"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="002C3E50"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -62,18 +52,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -439,74 +420,975 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Proyeccion de Costos - DataKnow</t>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Proyeccion</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>IC 95% Inf</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>IC 95% Sup</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Metodo</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Equipo 1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>$461.31</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>$443.00</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>$479.62</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Naive + Regresion Y</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Equipo 2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>$923.57</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>$889.75</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>$957.39</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Naive + Regresion Y+Z</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Price_Equipo1</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Proy_Equipo1</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Price_Equipo2</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Proy_Equipo2</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Price_Y</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Price_Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="n">
+        <v>45138</v>
+      </c>
+      <c r="B2" t="n">
+        <v>490.66</v>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="n">
+        <v>938.51</v>
+      </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="n">
+        <v>575</v>
+      </c>
+      <c r="G2" t="n">
+        <v>2195.25</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="n">
+        <v>45139</v>
+      </c>
+      <c r="B3" t="n">
+        <v>475.98</v>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="n">
+        <v>955.85</v>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="n">
+        <v>575</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2216.5</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="n">
+        <v>45140</v>
+      </c>
+      <c r="B4" t="n">
+        <v>482.49</v>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="n">
+        <v>945.28</v>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="n">
+        <v>570</v>
+      </c>
+      <c r="G4" t="n">
+        <v>2176.25</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="n">
+        <v>45141</v>
+      </c>
+      <c r="B5" t="n">
+        <v>455.93</v>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="n">
+        <v>941.11</v>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="n">
+        <v>564</v>
+      </c>
+      <c r="G5" t="n">
+        <v>2146.75</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="n">
+        <v>45142</v>
+      </c>
+      <c r="B6" t="n">
+        <v>467.25</v>
+      </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="n">
+        <v>955.87</v>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="n">
+        <v>568.33</v>
+      </c>
+      <c r="G6" t="n">
+        <v>2165</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="n">
+        <v>45145</v>
+      </c>
+      <c r="B7" t="n">
+        <v>459.48</v>
+      </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="n">
+        <v>937.85</v>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="n">
+        <v>568.33</v>
+      </c>
+      <c r="G7" t="n">
+        <v>2177.75</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="n">
+        <v>45146</v>
+      </c>
+      <c r="B8" t="n">
+        <v>485.36</v>
+      </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="n">
+        <v>940.5</v>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="n">
+        <v>568.33</v>
+      </c>
+      <c r="G8" t="n">
+        <v>2142.5</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="n">
+        <v>45147</v>
+      </c>
+      <c r="B9" t="n">
+        <v>478.44</v>
+      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="n">
+        <v>915.42</v>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="n">
+        <v>565</v>
+      </c>
+      <c r="G9" t="n">
+        <v>2152.5</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="n">
+        <v>45148</v>
+      </c>
+      <c r="B10" t="n">
+        <v>476.49</v>
+      </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="n">
+        <v>960.75</v>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="n">
+        <v>561.67</v>
+      </c>
+      <c r="G10" t="n">
+        <v>2161.25</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="n">
+        <v>45149</v>
+      </c>
+      <c r="B11" t="n">
+        <v>477.59</v>
+      </c>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="n">
+        <v>917.78</v>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="n">
+        <v>560</v>
+      </c>
+      <c r="G11" t="n">
+        <v>2126</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="n">
+        <v>45152</v>
+      </c>
+      <c r="B12" t="n">
+        <v>449.76</v>
+      </c>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="n">
+        <v>924.88</v>
+      </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="n">
+        <v>555</v>
+      </c>
+      <c r="G12" t="n">
+        <v>2095.75</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="n">
+        <v>45153</v>
+      </c>
+      <c r="B13" t="n">
+        <v>457.81</v>
+      </c>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="n">
+        <v>882.24</v>
+      </c>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="n">
+        <v>555</v>
+      </c>
+      <c r="G13" t="n">
+        <v>2085.25</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="n">
+        <v>45154</v>
+      </c>
+      <c r="B14" t="n">
+        <v>448.83</v>
+      </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="n">
+        <v>892.99</v>
+      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="n">
+        <v>555</v>
+      </c>
+      <c r="G14" t="n">
+        <v>2088.75</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="n">
+        <v>45155</v>
+      </c>
+      <c r="B15" t="n">
+        <v>447.58</v>
+      </c>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="n">
+        <v>920.27</v>
+      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="n">
+        <v>548.33</v>
+      </c>
+      <c r="G15" t="n">
+        <v>2130.5</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="n">
+        <v>45156</v>
+      </c>
+      <c r="B16" t="n">
+        <v>445.6</v>
+      </c>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="n">
+        <v>929.14</v>
+      </c>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="n">
+        <v>545</v>
+      </c>
+      <c r="G16" t="n">
+        <v>2095.75</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="n">
+        <v>45159</v>
+      </c>
+      <c r="B17" t="n">
+        <v>452.05</v>
+      </c>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="n">
+        <v>900.71</v>
+      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="n">
+        <v>545</v>
+      </c>
+      <c r="G17" t="n">
+        <v>2068.25</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="n">
+        <v>45160</v>
+      </c>
+      <c r="B18" t="n">
+        <v>446.52</v>
+      </c>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="n">
+        <v>940.41</v>
+      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="n">
+        <v>545</v>
+      </c>
+      <c r="G18" t="n">
+        <v>2121.25</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="n">
+        <v>45161</v>
+      </c>
+      <c r="B19" t="n">
+        <v>449.61</v>
+      </c>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="n">
+        <v>921.42</v>
+      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="n">
+        <v>555</v>
+      </c>
+      <c r="G19" t="n">
+        <v>2128.75</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="n">
+        <v>45162</v>
+      </c>
+      <c r="B20" t="n">
+        <v>450.7</v>
+      </c>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="n">
+        <v>918.34</v>
+      </c>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="n">
+        <v>554</v>
+      </c>
+      <c r="G20" t="n">
+        <v>2119.25</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="n">
+        <v>45163</v>
+      </c>
+      <c r="B21" t="n">
+        <v>450.36</v>
+      </c>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="n">
+        <v>899.65</v>
+      </c>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="n">
+        <v>554</v>
+      </c>
+      <c r="G21" t="n">
+        <v>2123.5</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="n">
+        <v>45166</v>
+      </c>
+      <c r="B22" t="n">
+        <v>469.03</v>
+      </c>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="n">
+        <v>933.2</v>
+      </c>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="n">
+        <v>549</v>
+      </c>
+      <c r="G22" t="n">
+        <v>2116.25</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="n">
+        <v>45167</v>
+      </c>
+      <c r="B23" t="n">
+        <v>460.42</v>
+      </c>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="n">
+        <v>901.79</v>
+      </c>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="n">
+        <v>545.33</v>
+      </c>
+      <c r="G23" t="n">
+        <v>2116.25</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="n">
+        <v>45168</v>
+      </c>
+      <c r="B24" t="n">
+        <v>464.8</v>
+      </c>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="n">
+        <v>945.4</v>
+      </c>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="n">
+        <v>543.67</v>
+      </c>
+      <c r="G24" t="n">
+        <v>2140.25</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="n">
+        <v>45169</v>
+      </c>
+      <c r="B25" t="n">
+        <v>451.73</v>
+      </c>
+      <c r="C25" t="n">
+        <v>461.3096958138468</v>
+      </c>
+      <c r="D25" t="n">
+        <v>955.35</v>
+      </c>
+      <c r="E25" t="n">
+        <v>923.5723004535308</v>
+      </c>
+      <c r="F25" t="n">
+        <v>545</v>
+      </c>
+      <c r="G25" t="n">
+        <v>2165.25</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Equipo</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Proyeccion</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>IC95% Inf</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>IC95% Sup</t>
-        </is>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Ecuacion</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Coeficiente</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>p-value</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Significancia</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>R²</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>MAE</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Std_Error</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Observaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Equipo 1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Price = 0.82 * Y + 5.56</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>const</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>5.5646</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>0.0000</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>***</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>0.9932</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>$7.64</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>$9.34</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>3530</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Equipo 1</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Price = 0.82 * Y + 5.56</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Price_Y</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>0.8181</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>0.0000</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>***</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>0.9932</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>$7.64</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>$9.34</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>3530</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Equipo 1</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="n">
-        <v>461.31</v>
-      </c>
-      <c r="C4" s="4" t="n">
-        <v>443</v>
-      </c>
-      <c r="D4" s="4" t="n">
-        <v>479.62</v>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Equipo 2</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Price = 0.36 * Y + 0.34 * Z + 7.02</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>const</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>7.022</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>0.0000</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>***</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>0.9898</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>$14.40</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>$17.26</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>3530</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Equipo 2</t>
         </is>
       </c>
-      <c r="B5" s="4" t="n">
-        <v>923.5700000000001</v>
-      </c>
-      <c r="C5" s="4" t="n">
-        <v>889.75</v>
-      </c>
-      <c r="D5" s="4" t="n">
-        <v>957.39</v>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Price = 0.36 * Y + 0.34 * Z + 7.02</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Price_Y</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>0.3552</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>0.0000</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>***</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>0.9898</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>$14.40</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>$17.26</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>3530</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Equipo 2</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Price = 0.36 * Y + 0.34 * Z + 7.02</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Price_Z</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>0.3365</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>0.0000</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>***</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>0.9898</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>$14.40</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>$17.26</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>3530</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Valor utilizado (Naive)</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Periodo referencia</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Metodo</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>$557.08</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2023-07-31 a 2023-08-31</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Media del ultimo mes</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>$2135.61</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2023-07-31 a 2023-08-31</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Media del ultimo mes</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>